<commit_message>
📊 Consolidated Test Report – Build #4 5d20adcd54f14c42103f45118154a8193df7c493
</commit_message>
<xml_diff>
--- a/security-reports/findings.xlsx
+++ b/security-reports/findings.xlsx
@@ -283,13 +283,13 @@
     <t>Assessment Date</t>
   </si>
   <si>
-    <t>2026-06-18 11:51:46 UTC</t>
+    <t>2026-06-18 12:25:41 UTC</t>
   </si>
   <si>
     <t>Build Number</t>
   </si>
   <si>
-    <t>3</t>
+    <t>4</t>
   </si>
   <si>
     <t>Total Security Rules Checked</t>

</xml_diff>

<commit_message>
📊 Consolidated Test Report – Build #5 3f6a3f329c10655459c2d42fad6114cbd5645977
</commit_message>
<xml_diff>
--- a/security-reports/findings.xlsx
+++ b/security-reports/findings.xlsx
@@ -283,13 +283,13 @@
     <t>Assessment Date</t>
   </si>
   <si>
-    <t>2026-06-18 12:25:41 UTC</t>
+    <t>2026-06-18 13:08:37 UTC</t>
   </si>
   <si>
     <t>Build Number</t>
   </si>
   <si>
-    <t>4</t>
+    <t>5</t>
   </si>
   <si>
     <t>Total Security Rules Checked</t>

</xml_diff>

<commit_message>
📊 Consolidated Test Report – Build #6 0d99462397ee5d74d9fe21b197429bb9627330ef
</commit_message>
<xml_diff>
--- a/security-reports/findings.xlsx
+++ b/security-reports/findings.xlsx
@@ -283,13 +283,13 @@
     <t>Assessment Date</t>
   </si>
   <si>
-    <t>2026-06-18 13:08:37 UTC</t>
+    <t>2026-06-18 13:36:08 UTC</t>
   </si>
   <si>
     <t>Build Number</t>
   </si>
   <si>
-    <t>5</t>
+    <t>6</t>
   </si>
   <si>
     <t>Total Security Rules Checked</t>

</xml_diff>

<commit_message>
📊 Consolidated Test Report – Build #7 b00dbddf9e82d71e4212189f6662a2085bfbe137
</commit_message>
<xml_diff>
--- a/security-reports/findings.xlsx
+++ b/security-reports/findings.xlsx
@@ -283,13 +283,13 @@
     <t>Assessment Date</t>
   </si>
   <si>
-    <t>2026-06-18 13:36:08 UTC</t>
+    <t>2026-06-18 14:09:54 UTC</t>
   </si>
   <si>
     <t>Build Number</t>
   </si>
   <si>
-    <t>6</t>
+    <t>7</t>
   </si>
   <si>
     <t>Total Security Rules Checked</t>

</xml_diff>

<commit_message>
📊 Consolidated Test Report – Build #8 ce181533a4ccc9db6b472b206f66e4f19253d3d4
</commit_message>
<xml_diff>
--- a/security-reports/findings.xlsx
+++ b/security-reports/findings.xlsx
@@ -283,13 +283,13 @@
     <t>Assessment Date</t>
   </si>
   <si>
-    <t>2026-06-18 14:09:54 UTC</t>
+    <t>2026-06-18 17:47:53 UTC</t>
   </si>
   <si>
     <t>Build Number</t>
   </si>
   <si>
-    <t>7</t>
+    <t>8</t>
   </si>
   <si>
     <t>Total Security Rules Checked</t>

</xml_diff>

<commit_message>
📊 Consolidated Test Report – Build #9 6000fae330714175134a377e8c3d08a2d82a3ecc
</commit_message>
<xml_diff>
--- a/security-reports/findings.xlsx
+++ b/security-reports/findings.xlsx
@@ -283,13 +283,13 @@
     <t>Assessment Date</t>
   </si>
   <si>
-    <t>2026-06-18 17:47:53 UTC</t>
+    <t>2026-06-19 06:37:38 UTC</t>
   </si>
   <si>
     <t>Build Number</t>
   </si>
   <si>
-    <t>8</t>
+    <t>9</t>
   </si>
   <si>
     <t>Total Security Rules Checked</t>

</xml_diff>

<commit_message>
📊 Consolidated Test Report – Build #10 47fdd5dc22e69507183db17eb0ab07bceeddd91a
</commit_message>
<xml_diff>
--- a/security-reports/findings.xlsx
+++ b/security-reports/findings.xlsx
@@ -283,13 +283,13 @@
     <t>Assessment Date</t>
   </si>
   <si>
-    <t>2026-06-19 06:37:38 UTC</t>
+    <t>2026-06-19 07:01:21 UTC</t>
   </si>
   <si>
     <t>Build Number</t>
   </si>
   <si>
-    <t>9</t>
+    <t>10</t>
   </si>
   <si>
     <t>Total Security Rules Checked</t>

</xml_diff>

<commit_message>
📊 Consolidated Test Report – Build #11 62fae82c26a2849d145da1721bc7b742fef7f045
</commit_message>
<xml_diff>
--- a/security-reports/findings.xlsx
+++ b/security-reports/findings.xlsx
@@ -283,13 +283,13 @@
     <t>Assessment Date</t>
   </si>
   <si>
-    <t>2026-06-19 07:01:21 UTC</t>
+    <t>2026-06-19 08:52:59 UTC</t>
   </si>
   <si>
     <t>Build Number</t>
   </si>
   <si>
-    <t>10</t>
+    <t>11</t>
   </si>
   <si>
     <t>Total Security Rules Checked</t>

</xml_diff>

<commit_message>
📊 Consolidated Test Report – Build #12 b62d184392af882a952387eba2a5cd4378cd0c48
</commit_message>
<xml_diff>
--- a/security-reports/findings.xlsx
+++ b/security-reports/findings.xlsx
@@ -283,13 +283,13 @@
     <t>Assessment Date</t>
   </si>
   <si>
-    <t>2026-06-19 08:52:59 UTC</t>
+    <t>2026-06-19 12:37:03 UTC</t>
   </si>
   <si>
     <t>Build Number</t>
   </si>
   <si>
-    <t>11</t>
+    <t>12</t>
   </si>
   <si>
     <t>Total Security Rules Checked</t>

</xml_diff>

<commit_message>
📊 Consolidated Test Report – Build #13 b422545380be0ff8c7ea02dc2966a4ddc02a308a
</commit_message>
<xml_diff>
--- a/security-reports/findings.xlsx
+++ b/security-reports/findings.xlsx
@@ -283,13 +283,13 @@
     <t>Assessment Date</t>
   </si>
   <si>
-    <t>2026-06-19 12:37:03 UTC</t>
+    <t>2026-06-20 07:19:01 UTC</t>
   </si>
   <si>
     <t>Build Number</t>
   </si>
   <si>
-    <t>12</t>
+    <t>13</t>
   </si>
   <si>
     <t>Total Security Rules Checked</t>

</xml_diff>

<commit_message>
📊 Consolidated Test Report – Build #14 8238c5fbc8d69b1411d3e0141b922b70619d116f
</commit_message>
<xml_diff>
--- a/security-reports/findings.xlsx
+++ b/security-reports/findings.xlsx
@@ -283,13 +283,13 @@
     <t>Assessment Date</t>
   </si>
   <si>
-    <t>2026-06-20 07:19:01 UTC</t>
+    <t>2026-06-20 07:42:47 UTC</t>
   </si>
   <si>
     <t>Build Number</t>
   </si>
   <si>
-    <t>13</t>
+    <t>14</t>
   </si>
   <si>
     <t>Total Security Rules Checked</t>

</xml_diff>

<commit_message>
📊 Consolidated Test Report – Build #15 d5eac3444f948c9cc376d6fa53139b7798dec008
</commit_message>
<xml_diff>
--- a/security-reports/findings.xlsx
+++ b/security-reports/findings.xlsx
@@ -283,13 +283,13 @@
     <t>Assessment Date</t>
   </si>
   <si>
-    <t>2026-06-20 07:42:47 UTC</t>
+    <t>2026-06-21 10:30:48 UTC</t>
   </si>
   <si>
     <t>Build Number</t>
   </si>
   <si>
-    <t>14</t>
+    <t>15</t>
   </si>
   <si>
     <t>Total Security Rules Checked</t>

</xml_diff>

<commit_message>
📊 Consolidated Test Report – Build #16 af4ef3bc176b878690d1f4b1a8af0ab0028f5e5f
</commit_message>
<xml_diff>
--- a/security-reports/findings.xlsx
+++ b/security-reports/findings.xlsx
@@ -283,13 +283,13 @@
     <t>Assessment Date</t>
   </si>
   <si>
-    <t>2026-06-21 10:30:48 UTC</t>
+    <t>2026-06-22 03:58:38 UTC</t>
   </si>
   <si>
     <t>Build Number</t>
   </si>
   <si>
-    <t>15</t>
+    <t>16</t>
   </si>
   <si>
     <t>Total Security Rules Checked</t>

</xml_diff>

<commit_message>
📊 Consolidated Test Report – Build #17 76c5c69c864d02f52c201e15b775f16c968b7404
</commit_message>
<xml_diff>
--- a/security-reports/findings.xlsx
+++ b/security-reports/findings.xlsx
@@ -283,13 +283,13 @@
     <t>Assessment Date</t>
   </si>
   <si>
-    <t>2026-06-22 03:58:38 UTC</t>
+    <t>2026-06-22 04:41:09 UTC</t>
   </si>
   <si>
     <t>Build Number</t>
   </si>
   <si>
-    <t>16</t>
+    <t>17</t>
   </si>
   <si>
     <t>Total Security Rules Checked</t>

</xml_diff>

<commit_message>
📊 Consolidated Test Report – Build #18 8771cc8b5e5eef1085c6bbef316d63a93e2d634f
</commit_message>
<xml_diff>
--- a/security-reports/findings.xlsx
+++ b/security-reports/findings.xlsx
@@ -283,13 +283,13 @@
     <t>Assessment Date</t>
   </si>
   <si>
-    <t>2026-06-22 04:41:09 UTC</t>
+    <t>2026-06-22 05:59:17 UTC</t>
   </si>
   <si>
     <t>Build Number</t>
   </si>
   <si>
-    <t>17</t>
+    <t>18</t>
   </si>
   <si>
     <t>Total Security Rules Checked</t>

</xml_diff>

<commit_message>
📊 Consolidated Test Report – Build #19 41823e6305917b74897985cd263ab51fd6abb7b3
</commit_message>
<xml_diff>
--- a/security-reports/findings.xlsx
+++ b/security-reports/findings.xlsx
@@ -283,13 +283,13 @@
     <t>Assessment Date</t>
   </si>
   <si>
-    <t>2026-06-22 05:59:17 UTC</t>
+    <t>2026-06-22 06:47:02 UTC</t>
   </si>
   <si>
     <t>Build Number</t>
   </si>
   <si>
-    <t>18</t>
+    <t>19</t>
   </si>
   <si>
     <t>Total Security Rules Checked</t>

</xml_diff>

<commit_message>
📊 Consolidated Test Report – Build #20 1a271675ddf3a3067ebaf6bd5e93729ea56bea9d
</commit_message>
<xml_diff>
--- a/security-reports/findings.xlsx
+++ b/security-reports/findings.xlsx
@@ -283,13 +283,13 @@
     <t>Assessment Date</t>
   </si>
   <si>
-    <t>2026-06-22 06:47:02 UTC</t>
+    <t>2026-06-22 07:27:47 UTC</t>
   </si>
   <si>
     <t>Build Number</t>
   </si>
   <si>
-    <t>19</t>
+    <t>20</t>
   </si>
   <si>
     <t>Total Security Rules Checked</t>

</xml_diff>

<commit_message>
📊 Consolidated Test Report – Build #21 92cb00e1a85a4b49f320527f16cb21d33a4e5ac6
</commit_message>
<xml_diff>
--- a/security-reports/findings.xlsx
+++ b/security-reports/findings.xlsx
@@ -283,13 +283,13 @@
     <t>Assessment Date</t>
   </si>
   <si>
-    <t>2026-06-22 07:27:47 UTC</t>
+    <t>2026-06-22 08:31:20 UTC</t>
   </si>
   <si>
     <t>Build Number</t>
   </si>
   <si>
-    <t>20</t>
+    <t>21</t>
   </si>
   <si>
     <t>Total Security Rules Checked</t>

</xml_diff>

<commit_message>
📊 Consolidated Test Report – Build #22 0705567c07530bda180e09603cd2b77619736113
</commit_message>
<xml_diff>
--- a/security-reports/findings.xlsx
+++ b/security-reports/findings.xlsx
@@ -283,13 +283,13 @@
     <t>Assessment Date</t>
   </si>
   <si>
-    <t>2026-06-22 08:31:20 UTC</t>
+    <t>2026-06-22 09:17:50 UTC</t>
   </si>
   <si>
     <t>Build Number</t>
   </si>
   <si>
-    <t>21</t>
+    <t>22</t>
   </si>
   <si>
     <t>Total Security Rules Checked</t>

</xml_diff>

<commit_message>
📊 Consolidated Test Report – Build #23 92cd199b98e50663c4bfe526ecdafa0a624cfb63
</commit_message>
<xml_diff>
--- a/security-reports/findings.xlsx
+++ b/security-reports/findings.xlsx
@@ -283,13 +283,13 @@
     <t>Assessment Date</t>
   </si>
   <si>
-    <t>2026-06-22 09:17:50 UTC</t>
+    <t>2026-06-22 10:09:12 UTC</t>
   </si>
   <si>
     <t>Build Number</t>
   </si>
   <si>
-    <t>22</t>
+    <t>23</t>
   </si>
   <si>
     <t>Total Security Rules Checked</t>

</xml_diff>

<commit_message>
📊 Consolidated Test Report – Build #24 ad117b39c7d0799d3774b0a560eb99201fe6752d
</commit_message>
<xml_diff>
--- a/security-reports/findings.xlsx
+++ b/security-reports/findings.xlsx
@@ -283,13 +283,13 @@
     <t>Assessment Date</t>
   </si>
   <si>
-    <t>2026-06-22 10:09:12 UTC</t>
+    <t>2026-06-22 11:55:55 UTC</t>
   </si>
   <si>
     <t>Build Number</t>
   </si>
   <si>
-    <t>23</t>
+    <t>24</t>
   </si>
   <si>
     <t>Total Security Rules Checked</t>

</xml_diff>

<commit_message>
📊 Consolidated Test Report – Build #25 d4df82df77ec342dfc19fd5dd53415e8980cbe95
</commit_message>
<xml_diff>
--- a/security-reports/findings.xlsx
+++ b/security-reports/findings.xlsx
@@ -283,13 +283,13 @@
     <t>Assessment Date</t>
   </si>
   <si>
-    <t>2026-06-22 11:55:55 UTC</t>
+    <t>2026-06-22 12:29:25 UTC</t>
   </si>
   <si>
     <t>Build Number</t>
   </si>
   <si>
-    <t>24</t>
+    <t>25</t>
   </si>
   <si>
     <t>Total Security Rules Checked</t>

</xml_diff>

<commit_message>
📊 Consolidated Test Report – Build #26 df071f5b01d9100774598c845989586255e63cbd
</commit_message>
<xml_diff>
--- a/security-reports/findings.xlsx
+++ b/security-reports/findings.xlsx
@@ -283,13 +283,13 @@
     <t>Assessment Date</t>
   </si>
   <si>
-    <t>2026-06-22 12:29:25 UTC</t>
+    <t>2026-06-22 13:00:51 UTC</t>
   </si>
   <si>
     <t>Build Number</t>
   </si>
   <si>
-    <t>25</t>
+    <t>26</t>
   </si>
   <si>
     <t>Total Security Rules Checked</t>

</xml_diff>

<commit_message>
📊 Consolidated Test Report – Build #27 f1675b5f26ae1a371e8d56ccfb9a1e4a0d2f16a0
</commit_message>
<xml_diff>
--- a/security-reports/findings.xlsx
+++ b/security-reports/findings.xlsx
@@ -283,13 +283,13 @@
     <t>Assessment Date</t>
   </si>
   <si>
-    <t>2026-06-22 13:00:51 UTC</t>
+    <t>2026-06-22 13:42:36 UTC</t>
   </si>
   <si>
     <t>Build Number</t>
   </si>
   <si>
-    <t>26</t>
+    <t>27</t>
   </si>
   <si>
     <t>Total Security Rules Checked</t>

</xml_diff>

<commit_message>
📊 Consolidated Test Report – Build #28 db98f361294517f59fc7e9bc4987ed69e97e0bc9
</commit_message>
<xml_diff>
--- a/security-reports/findings.xlsx
+++ b/security-reports/findings.xlsx
@@ -283,13 +283,13 @@
     <t>Assessment Date</t>
   </si>
   <si>
-    <t>2026-06-22 13:42:36 UTC</t>
+    <t>2026-06-22 14:18:00 UTC</t>
   </si>
   <si>
     <t>Build Number</t>
   </si>
   <si>
-    <t>27</t>
+    <t>28</t>
   </si>
   <si>
     <t>Total Security Rules Checked</t>

</xml_diff>

<commit_message>
📊 Consolidated Test Report – Build #29 ce98edcd5e2d18b7f195b5c9464c1bb9e3b48d9b
</commit_message>
<xml_diff>
--- a/security-reports/findings.xlsx
+++ b/security-reports/findings.xlsx
@@ -283,13 +283,13 @@
     <t>Assessment Date</t>
   </si>
   <si>
-    <t>2026-06-22 14:18:00 UTC</t>
+    <t>2026-06-22 14:41:32 UTC</t>
   </si>
   <si>
     <t>Build Number</t>
   </si>
   <si>
-    <t>28</t>
+    <t>29</t>
   </si>
   <si>
     <t>Total Security Rules Checked</t>

</xml_diff>

<commit_message>
📊 Consolidated Test Report – Build #30 78de3f5fb8f788db1c64f2a262b233af419c90ce
</commit_message>
<xml_diff>
--- a/security-reports/findings.xlsx
+++ b/security-reports/findings.xlsx
@@ -283,13 +283,13 @@
     <t>Assessment Date</t>
   </si>
   <si>
-    <t>2026-06-22 14:41:32 UTC</t>
+    <t>2026-06-22 16:48:58 UTC</t>
   </si>
   <si>
     <t>Build Number</t>
   </si>
   <si>
-    <t>29</t>
+    <t>30</t>
   </si>
   <si>
     <t>Total Security Rules Checked</t>

</xml_diff>

<commit_message>
📊 Consolidated Test Report – Build #31 83e96d472c27c5b3099c6583c7768b0d72831eca
</commit_message>
<xml_diff>
--- a/security-reports/findings.xlsx
+++ b/security-reports/findings.xlsx
@@ -283,13 +283,13 @@
     <t>Assessment Date</t>
   </si>
   <si>
-    <t>2026-06-22 16:48:58 UTC</t>
+    <t>2026-06-23 07:45:09 UTC</t>
   </si>
   <si>
     <t>Build Number</t>
   </si>
   <si>
-    <t>30</t>
+    <t>31</t>
   </si>
   <si>
     <t>Total Security Rules Checked</t>

</xml_diff>